<commit_message>
Culminado para la desicion de contrato
</commit_message>
<xml_diff>
--- a/Resultados_datos_afiliados.xlsx
+++ b/Resultados_datos_afiliados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,27 +439,32 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>IPS Primaria</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tipo Contrato</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Departamento</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Municipio</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tipo Afiliado</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Categoría Afiliado</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>IPS Primaria</t>
         </is>
       </c>
     </row>
@@ -469,8 +474,10 @@
           <t>RC</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1055274915</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1055274915_x000d_</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
@@ -479,10 +486,15 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -490,8 +502,10 @@
           <t>TI</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>1011210568</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1011210568_x000d_</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -503,27 +517,32 @@
           <t>CANCELADO</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>BOYACA</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>TUNJA</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>BENEFICIARIOS</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -531,8 +550,10 @@
           <t>CC</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>12658</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12658_x000d_</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -546,27 +567,32 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>SERVICIOS MEDICOS FAMEDIC S.A.S-DUITAMA</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PGP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>BOYACA</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>DUITAMA</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>CABEZA DE FAMILIA</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>SERVICIOS MEDICOS FAMEDIC S.A.S-DUITAMA</t>
         </is>
       </c>
     </row>
@@ -576,8 +602,10 @@
           <t>CC</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>9513594</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>9513594_x000d_</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -591,27 +619,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>SERVICIOS MEDICOS FAMEDIC S.A.S-DUITAMA</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PGP</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>BOYACA</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>TIBASOSA</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>CABEZA DE FAMILIA</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>SERVICIOS MEDICOS FAMEDIC S.A.S-DUITAMA</t>
         </is>
       </c>
     </row>
@@ -621,8 +654,10 @@
           <t>CC</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>23556241</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>23556241_x000d_</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -634,27 +669,392 @@
           <t>CANCELADO</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>BOYACA</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>DUITAMA</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>SEGUNDOS COTIZANTES</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>19082926_x000d_</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>JORGE AUGUSTO TELLEZ GOMEZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>E.S.E. HOSPITAL JOSE CAYETANO VASQUEZ - CAPITA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PUERTO BOYACA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BENEFICIARIOS</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>9511215_x000d_</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PEDRO ARTURO RODRIGUEZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CANCELADO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CHIQUINQUIRA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1053348031_x000d_</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DUVAN JAIR NIETO RAMIREZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CENTRO MEDICO COLSUBSIDIO CHIQUINQUIRA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PGP</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>CHIQUINQUIRA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4264656_x000d_</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>JOSE ESTEBAN GRANADOS MORALES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SERVICIOS INTEGRALES DE REHABILITACION EN BOYACA LIMITADA- SIREB LTDA SEDE PAIPA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PAIPA</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20161653_x000d_</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SUSANA AVELLA JIMENEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SERVICIOS MEDICOS FAMEDIC S.A.S-DUITAMA</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PGP</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>DUITAMA</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CC_x000d_</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>23485006_x000d_</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MARIA BELLABEL TORRES CRISTANCHO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CENTRO MEDICO COLSUBSIDIO CHIQUINQUIRA</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PGP</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>CHIQUINQUIRA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>74130336</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MIGUEL ALEXANDER VELANDIA SANCHEZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SERVICIOS INTEGRALES DE REHABILITACION EN BOYACA LIMITADA- SIREB LTDA SEDE PAIPA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>EVENTO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BOYACA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PAIPA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CABEZA DE FAMILIA</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>